<commit_message>
*timesreport.gms* Minor change to definition of vintage (now subset of allyear) + adjusted import of levelized costs so that they second dimension imported is now vintage. *Scen_Z_TIMESReport.xlsx* added RFCmd_F	$SET ANNCOST LE = 2 to ensure that costs are NOT accounted for in years before model horizont (BOH)
</commit_message>
<xml_diff>
--- a/SysSettings.xlsx
+++ b/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kristoffer\DemoS_012_timesreport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44BF8C9-638E-4891-80B8-CFF8F2772D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DEBF54-460E-4CC8-BBA5-1028F83563E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="853" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34670" yWindow="-110" windowWidth="34780" windowHeight="21100" tabRatio="853" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Region-Time Slices" sheetId="16" r:id="rId1"/>
@@ -211,7 +211,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="145">
   <si>
     <t>~TFM_UPD</t>
   </si>
@@ -615,9 +615,6 @@
     <t>Coal</t>
   </si>
   <si>
-    <t>TFM_INS</t>
-  </si>
-  <si>
     <t>NRG_BIO</t>
   </si>
   <si>
@@ -637,21 +634,41 @@
   </si>
   <si>
     <t>GHG-emission</t>
+  </si>
+  <si>
+    <t>Other_indexes</t>
+  </si>
+  <si>
+    <t>RFCmd_FLAGS</t>
+  </si>
+  <si>
+    <t>$SET MEMCLEAN NO</t>
+  </si>
+  <si>
+    <t>$SET ANNCOST LEV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="_([$€]* #,##0.00_);_([$€]* \(#,##0.00\);_([$€]* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -824,6 +841,12 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF404040"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1107,206 +1130,226 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="30">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment horizontal="left" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="4" fontId="23" fillId="11" borderId="3">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="23" fillId="11" borderId="3">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="17">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="4" fontId="24" fillId="0" borderId="0" applyBorder="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="4" fontId="24" fillId="0" borderId="3" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="4" fontId="24" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment horizontal="left" vertical="center" indent="5"/>
-    </xf>
-    <xf numFmtId="4" fontId="22" fillId="11" borderId="3">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="22" fillId="11" borderId="3">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="17">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="4" fontId="23" fillId="0" borderId="0" applyBorder="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="4" fontId="23" fillId="0" borderId="3" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="4" fontId="23" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="4" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="17" fillId="4" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="2" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="16" fillId="4" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="17" fillId="4" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="13" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="16" fillId="4" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="17" fillId="4" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="17" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="17" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="15" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="27"/>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" xfId="27" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="27"/>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="27" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="30"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="30" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="30" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="30" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="30">
+  <cellStyles count="43">
     <cellStyle name="5x indented GHG Textfiels" xfId="8" xr:uid="{E636D3A7-254D-4A7E-AE66-E5B25926F024}"/>
     <cellStyle name="AggOrange_CRFReport-template" xfId="9" xr:uid="{68131F4B-F2D7-4AF0-9C57-EE4BD427A2EF}"/>
     <cellStyle name="AggOrange9_CRFReport-template" xfId="10" xr:uid="{E0583BC3-B6E6-4778-BD53-CA75D9E52640}"/>
@@ -1318,18 +1361,31 @@
     <cellStyle name="Normal 10" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
     <cellStyle name="Normal 10 2" xfId="21" xr:uid="{E15E9843-3071-4157-A7C0-D2B2D8775015}"/>
     <cellStyle name="Normal 11" xfId="27" xr:uid="{8A6FC8E4-D04B-4D12-858A-9B467C5C2B68}"/>
+    <cellStyle name="Normal 11 2" xfId="38" xr:uid="{E4DFD373-11A3-4CD1-B6A0-F05DDB3180FA}"/>
+    <cellStyle name="Normal 12" xfId="34" xr:uid="{9D7D45DF-D40E-426C-8765-F319C53A65B7}"/>
+    <cellStyle name="Normal 12 2" xfId="41" xr:uid="{74E59AB7-5033-454E-8F11-D4642667F762}"/>
+    <cellStyle name="Normal 12 3" xfId="42" xr:uid="{5456D9F3-E0BC-4783-9D98-92426B8F4337}"/>
+    <cellStyle name="Normal 13" xfId="30" xr:uid="{B26ED7C7-768C-4F63-9F9F-CEDBA0F2A9D6}"/>
     <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Normal 3" xfId="14" xr:uid="{DE5F4A50-F6A3-4774-AF7D-4CE89FCC23DB}"/>
     <cellStyle name="Normal 3 2" xfId="26" xr:uid="{94B08955-980C-4264-AFCC-EA9F0C36CE97}"/>
+    <cellStyle name="Normal 3 2 2" xfId="37" xr:uid="{3A5CC4AB-F8F7-4E0F-A866-047446F41781}"/>
     <cellStyle name="Normal 3 3" xfId="29" xr:uid="{41D528A3-C845-406C-B7E8-F126A177976D}"/>
+    <cellStyle name="Normal 3 3 2" xfId="40" xr:uid="{A371384A-007D-4265-9406-D0CFADE1BEC4}"/>
+    <cellStyle name="Normal 3 4" xfId="31" xr:uid="{3BD09752-C5E1-45D9-B638-5DEC2B7B04DD}"/>
     <cellStyle name="Normal 4" xfId="15" xr:uid="{89F21CF0-5A68-411B-9ABF-5C16CA183596}"/>
     <cellStyle name="Normal 5" xfId="7" xr:uid="{6C48E7FE-F840-4FE5-A609-66FBBF550150}"/>
     <cellStyle name="Normal 5 2" xfId="25" xr:uid="{D4AA070D-0B50-4B0E-B3D8-FA429F7B588C}"/>
+    <cellStyle name="Normal 5 2 2" xfId="36" xr:uid="{40DD2FF1-5A95-4BCF-B09C-E02236888530}"/>
     <cellStyle name="Normal 5 3" xfId="28" xr:uid="{2FC0E98B-28BF-4FFC-A427-B1C13E6909CC}"/>
+    <cellStyle name="Normal 5 3 2" xfId="39" xr:uid="{30F57278-833F-406D-AAD0-805CDDC713C4}"/>
+    <cellStyle name="Normal 5 4" xfId="32" xr:uid="{6973B70F-65BF-4EAD-9C8B-DB8E43B7AA79}"/>
     <cellStyle name="Normal 6" xfId="22" xr:uid="{38799B17-C241-4FDA-B956-13B151EC805D}"/>
     <cellStyle name="Normal 7" xfId="23" xr:uid="{4CE8E9A5-D8F7-4EC9-8974-B63FF5910DCE}"/>
     <cellStyle name="Normal 8" xfId="6" xr:uid="{E32D2269-89F5-4B8D-B187-64D7F5EAA460}"/>
+    <cellStyle name="Normal 8 2" xfId="35" xr:uid="{E75746D3-7760-4689-8686-05A92BAC806F}"/>
     <cellStyle name="Normal 9" xfId="24" xr:uid="{9D2D5792-5B6A-43F0-9B6D-15F5A83BCF87}"/>
+    <cellStyle name="Normal 9 2" xfId="33" xr:uid="{C7881742-AE50-42D1-AD33-B84DE8C3B451}"/>
     <cellStyle name="Normal GHG Numbers (0.00)" xfId="16" xr:uid="{BAC52154-6D7C-4EFB-B85B-ED63E1A3D24A}"/>
     <cellStyle name="Normal GHG Textfiels Bold" xfId="17" xr:uid="{D1173938-2398-4A42-B395-C089D0A32E4D}"/>
     <cellStyle name="Normal GHG-Shade" xfId="18" xr:uid="{D39DB488-9AAC-4C16-9A10-35F7E9CA2B4A}"/>
@@ -3321,14 +3377,14 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>487680</xdr:colOff>
-      <xdr:row>3</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>45720</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
       <xdr:colOff>118588</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>29685</xdr:rowOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>36035</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -3787,16 +3843,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:J6"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.08984375" customWidth="1"/>
-    <col min="2" max="2" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6328125" customWidth="1"/>
-    <col min="7" max="7" width="3.36328125" customWidth="1"/>
-    <col min="8" max="8" width="29.36328125" customWidth="1"/>
+    <col min="1" max="1" width="2.140625" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="3.42578125" customWidth="1"/>
+    <col min="8" max="8" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3806,7 +3862,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="2:10" ht="13" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
@@ -3823,7 +3879,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B5" s="15" t="s">
         <v>54</v>
       </c>
@@ -3837,7 +3893,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B6" s="15" t="s">
         <v>83</v>
       </c>
@@ -3852,7 +3908,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -3864,42 +3920,42 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B3:D23"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.81640625" customWidth="1"/>
-    <col min="6" max="6" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4">
         <v>2005</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="65" t="s">
         <v>40</v>
       </c>
@@ -3910,7 +3966,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" s="14">
         <v>1</v>
       </c>
@@ -3921,7 +3977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" s="14">
         <v>2</v>
       </c>
@@ -3932,7 +3988,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" s="14"/>
       <c r="C15" s="14">
         <v>5</v>
@@ -3941,7 +3997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B16" s="14"/>
       <c r="C16" s="14">
         <v>5</v>
@@ -3950,7 +4006,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="14"/>
       <c r="C17" s="14">
         <v>5</v>
@@ -3959,42 +4015,42 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
       <c r="D22" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
       <c r="D23" s="14">
@@ -4002,7 +4058,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -4013,18 +4069,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B3:C11"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.36328125" customWidth="1"/>
-    <col min="2" max="2" width="52.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.42578125" customWidth="1"/>
+    <col min="2" max="2" width="52.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="2:3" ht="13" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="13" t="s">
         <v>32</v>
       </c>
@@ -4032,7 +4088,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="63" t="s">
         <v>34</v>
       </c>
@@ -4040,7 +4096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="14" t="s">
         <v>35</v>
       </c>
@@ -4048,7 +4104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="14" t="s">
         <v>36</v>
       </c>
@@ -4056,7 +4112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="14" t="s">
         <v>37</v>
       </c>
@@ -4064,7 +4120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="14" t="s">
         <v>98</v>
       </c>
@@ -4072,7 +4128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="14" t="s">
         <v>99</v>
       </c>
@@ -4080,7 +4136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="14" t="s">
         <v>85</v>
       </c>
@@ -4089,7 +4145,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -4100,23 +4156,23 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B3:Q36"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.81640625" customWidth="1"/>
-    <col min="4" max="4" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6328125" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.7265625" customWidth="1"/>
-    <col min="13" max="13" width="9.26953125" customWidth="1"/>
+    <col min="1" max="1" width="2.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" ht="13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>19</v>
       </c>
@@ -4136,7 +4192,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
         <v>86</v>
       </c>
@@ -4150,7 +4206,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>86</v>
       </c>
@@ -4164,7 +4220,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>86</v>
       </c>
@@ -4178,26 +4234,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="2:4" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="2:4" ht="15" x14ac:dyDescent="0.2">
       <c r="B30" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="2:4" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:4" ht="18" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
         <v>44</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
     </row>
-    <row r="33" spans="2:17" ht="13" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B33" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:17" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B34" s="5" t="s">
         <v>19</v>
       </c>
@@ -4247,7 +4303,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:17" x14ac:dyDescent="0.2">
       <c r="D35" t="s">
         <v>4</v>
       </c>
@@ -4261,7 +4317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:17" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
         <v>4</v>
       </c>
@@ -4287,28 +4343,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B3:H33"/>
-  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="10"/>
-    <col min="2" max="2" width="12.08984375" style="10" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" style="10" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="10"/>
+    <col min="2" max="2" width="12.140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" style="10" customWidth="1"/>
     <col min="4" max="4" width="14" style="10" customWidth="1"/>
-    <col min="5" max="5" width="10.36328125" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.36328125" style="10" customWidth="1"/>
-    <col min="7" max="16384" width="9.08984375" style="10"/>
+    <col min="5" max="5" width="10.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="10" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="10"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" ht="15" x14ac:dyDescent="0.2">
       <c r="B3" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="13" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B5" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>19</v>
       </c>
@@ -4331,7 +4387,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
       <c r="D7" s="10" t="s">
         <v>56</v>
       </c>
@@ -4339,7 +4395,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
       <c r="D8" s="10" t="s">
         <v>46</v>
       </c>
@@ -4347,7 +4403,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>63</v>
       </c>
@@ -4359,7 +4415,7 @@
         <v>0.24971461187214614</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B10" s="10" t="s">
         <v>64</v>
       </c>
@@ -4371,7 +4427,7 @@
         <v>0.22973744292237441</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B11" s="10" t="s">
         <v>65</v>
       </c>
@@ -4383,7 +4439,7 @@
         <v>0.24942922374429224</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
         <v>66</v>
       </c>
@@ -4395,7 +4451,7 @@
         <v>0.27111872146118721</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" s="10" t="s">
@@ -4411,34 +4467,34 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B14"/>
       <c r="C14"/>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B15"/>
       <c r="C15"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17"/>
       <c r="C17"/>
       <c r="D17"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18"/>
     </row>
-    <row r="19" spans="2:7" ht="17.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" ht="18" x14ac:dyDescent="0.25">
       <c r="B19" s="18" t="s">
         <v>62</v>
       </c>
@@ -4448,11 +4504,11 @@
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C20" s="21"/>
       <c r="D20" s="21"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="22" t="s">
         <v>21</v>
       </c>
@@ -4469,7 +4525,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="23" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" ht="24" x14ac:dyDescent="0.2">
       <c r="B22" s="26"/>
       <c r="C22" s="27" t="s">
         <v>67</v>
@@ -4484,7 +4540,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="22" t="s">
         <v>55</v>
       </c>
@@ -4509,14 +4565,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="34"/>
       <c r="C24" s="34"/>
       <c r="D24" s="34"/>
       <c r="E24" s="34"/>
       <c r="F24" s="34"/>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="34"/>
       <c r="C25" s="35"/>
       <c r="D25" s="35"/>
@@ -4524,7 +4580,7 @@
       <c r="F25" s="34"/>
       <c r="G25" s="34"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="34"/>
       <c r="C26" s="36" t="s">
         <v>71</v>
@@ -4538,7 +4594,7 @@
       <c r="F26" s="39"/>
       <c r="G26" s="34"/>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="40" t="s">
         <v>74</v>
       </c>
@@ -4555,7 +4611,7 @@
       <c r="F27" s="44"/>
       <c r="G27" s="34"/>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="45" t="s">
         <v>76</v>
       </c>
@@ -4573,7 +4629,7 @@
       <c r="F28" s="44"/>
       <c r="G28" s="34"/>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="34"/>
       <c r="C29" s="34"/>
       <c r="D29" s="49">
@@ -4587,7 +4643,7 @@
       <c r="F29" s="51"/>
       <c r="G29" s="34"/>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="34"/>
       <c r="C30" s="34"/>
       <c r="D30" s="52"/>
@@ -4595,7 +4651,7 @@
       <c r="F30" s="34"/>
       <c r="G30" s="34"/>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="53"/>
       <c r="C31" s="54" t="s">
         <v>78</v>
@@ -4607,7 +4663,7 @@
       <c r="F31" s="34"/>
       <c r="G31" s="34"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="56" t="s">
         <v>75</v>
       </c>
@@ -4624,7 +4680,7 @@
       </c>
       <c r="G32" s="34"/>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="59" t="s">
         <v>80</v>
       </c>
@@ -4653,17 +4709,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:I6"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" ht="13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>48</v>
       </c>
@@ -4671,7 +4727,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="13" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="11" t="s">
         <v>49</v>
       </c>
@@ -4694,7 +4750,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B4" s="15" t="s">
         <v>97</v>
       </c>
@@ -4717,7 +4773,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
       <c r="D5" t="s">
         <v>52</v>
       </c>
@@ -4737,7 +4793,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
       <c r="D6" t="s">
         <v>53</v>
       </c>
@@ -4767,18 +4823,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B2:L199"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.08984375" customWidth="1"/>
-    <col min="2" max="2" width="15.7265625" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
     <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="11.26953125" customWidth="1"/>
-    <col min="9" max="11" width="11.81640625" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.28515625" customWidth="1"/>
+    <col min="9" max="11" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:12" ht="15" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
         <v>41</v>
       </c>
@@ -4789,7 +4845,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
         <v>6</v>
       </c>
@@ -4798,12 +4854,12 @@
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
@@ -4823,7 +4879,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="27" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:12" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="70" t="s">
         <v>42</v>
       </c>
@@ -4844,7 +4900,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B8" t="str">
         <f t="shared" ref="B8:B13" si="0">IF(J8=0,"",J8)</f>
         <v>NRG_ELC</v>
@@ -4871,7 +4927,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="9" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>NRG_GAS</v>
@@ -4897,7 +4953,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>NRG_NUK</v>
@@ -4923,7 +4979,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="11" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>NRG_OIL</v>
@@ -4949,7 +5005,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="12" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>NRG_RNW</v>
@@ -4975,7 +5031,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="13" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>NRG_COA</v>
@@ -5001,7 +5057,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="14" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f t="shared" ref="B14:B72" si="3">IF(J14=0,"",J14)</f>
         <v>NRG_BIO</v>
@@ -5019,22 +5075,22 @@
         <v>y</v>
       </c>
       <c r="J14" s="71" t="s">
+        <v>134</v>
+      </c>
+      <c r="K14" s="71" t="s">
         <v>135</v>
-      </c>
-      <c r="K14" s="71" t="s">
-        <v>136</v>
       </c>
       <c r="L14" s="71" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f t="shared" si="3"/>
         <v>ENV_CO2</v>
       </c>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="5"/>
@@ -5045,16 +5101,16 @@
         <v>y</v>
       </c>
       <c r="J15" s="71" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="L15" s="71" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f t="shared" si="3"/>
         <v>DEM_COM</v>
@@ -5072,16 +5128,16 @@
         <v>y</v>
       </c>
       <c r="J16" s="71" t="s">
+        <v>138</v>
+      </c>
+      <c r="K16" s="71" t="s">
         <v>139</v>
-      </c>
-      <c r="K16" s="71" t="s">
-        <v>140</v>
       </c>
       <c r="L16" s="71" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5099,7 +5155,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5117,7 +5173,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5135,7 +5191,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5153,7 +5209,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5171,7 +5227,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5189,7 +5245,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5207,7 +5263,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5225,7 +5281,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5243,7 +5299,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5261,7 +5317,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5279,7 +5335,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5297,7 +5353,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5315,7 +5371,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5333,7 +5389,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5351,7 +5407,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5369,7 +5425,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5387,7 +5443,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5405,7 +5461,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5423,7 +5479,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5441,7 +5497,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5459,7 +5515,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B38" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5477,7 +5533,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5495,7 +5551,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5513,7 +5569,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5531,7 +5587,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5549,7 +5605,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5567,7 +5623,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B44" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5585,7 +5641,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5603,7 +5659,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5621,7 +5677,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5639,7 +5695,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5657,7 +5713,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B49" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5675,7 +5731,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B50" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5693,7 +5749,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B51" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5711,7 +5767,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B52" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5729,7 +5785,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B53" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5747,7 +5803,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B54" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5765,7 +5821,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B55" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5783,7 +5839,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B56" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5801,7 +5857,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B57" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5819,7 +5875,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B58" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5837,7 +5893,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B59" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5855,7 +5911,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B60" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5873,7 +5929,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B61" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5891,7 +5947,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B62" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5909,7 +5965,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B63" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5927,7 +5983,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B64" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5945,7 +6001,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B65" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5963,7 +6019,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B66" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5981,7 +6037,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B67" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5999,7 +6055,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B68" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6017,7 +6073,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B69" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6035,7 +6091,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B70" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6053,7 +6109,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B71" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6071,7 +6127,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B72" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6089,7 +6145,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B73" t="str">
         <f t="shared" ref="B73:B136" si="7">IF(J73=0,"",J73)</f>
         <v/>
@@ -6107,7 +6163,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B74" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6125,7 +6181,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B75" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6143,7 +6199,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B76" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6161,7 +6217,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B77" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6179,7 +6235,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B78" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6197,7 +6253,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B79" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6215,7 +6271,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B80" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6233,7 +6289,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B81" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6251,7 +6307,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B82" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6269,7 +6325,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B83" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6287,7 +6343,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B84" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6305,7 +6361,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B85" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6323,7 +6379,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B86" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6341,7 +6397,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B87" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6359,7 +6415,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B88" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6377,7 +6433,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B89" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6395,7 +6451,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B90" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6413,7 +6469,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B91" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6431,7 +6487,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B92" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6449,7 +6505,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B93" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6467,7 +6523,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B94" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6485,7 +6541,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B95" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6503,7 +6559,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B96" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6521,7 +6577,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B97" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6539,7 +6595,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B98" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6557,7 +6613,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B99" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6575,7 +6631,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B100" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6593,7 +6649,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B101" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6611,7 +6667,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B102" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6629,7 +6685,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B103" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6647,7 +6703,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B104" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6665,7 +6721,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B105" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6683,7 +6739,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B106" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6701,7 +6757,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B107" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6719,7 +6775,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B108" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6737,7 +6793,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B109" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6755,7 +6811,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B110" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6773,7 +6829,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B111" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6791,7 +6847,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B112" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6809,7 +6865,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B113" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6827,7 +6883,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B114" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6845,7 +6901,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B115" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6863,7 +6919,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B116" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6881,7 +6937,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B117" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6899,7 +6955,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B118" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6917,7 +6973,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B119" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6935,7 +6991,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B120" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6953,7 +7009,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B121" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6971,7 +7027,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B122" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6989,7 +7045,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B123" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7007,7 +7063,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B124" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7025,7 +7081,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B125" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7043,7 +7099,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B126" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7061,7 +7117,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B127" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7079,7 +7135,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B128" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7097,7 +7153,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B129" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7115,7 +7171,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B130" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7133,7 +7189,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B131" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7151,7 +7207,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B132" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7169,7 +7225,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B133" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7187,7 +7243,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B134" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7205,7 +7261,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B135" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7223,7 +7279,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B136" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7241,7 +7297,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B137" t="str">
         <f t="shared" ref="B137:B198" si="11">IF(J137=0,"",J137)</f>
         <v/>
@@ -7259,7 +7315,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B138" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7277,7 +7333,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B139" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7295,7 +7351,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B140" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7313,7 +7369,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B141" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7331,7 +7387,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B142" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7349,7 +7405,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B143" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7367,7 +7423,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B144" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7385,7 +7441,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B145" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7403,7 +7459,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B146" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7421,7 +7477,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B147" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7439,7 +7495,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B148" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7457,7 +7513,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B149" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7475,7 +7531,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B150" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7493,7 +7549,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B151" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7511,7 +7567,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B152" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7529,7 +7585,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B153" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7547,7 +7603,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B154" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7565,7 +7621,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B155" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7583,7 +7639,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B156" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7601,7 +7657,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B157" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7619,7 +7675,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B158" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7637,7 +7693,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B159" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7655,7 +7711,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B160" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7673,7 +7729,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B161" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7691,7 +7747,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B162" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7709,7 +7765,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B163" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7727,7 +7783,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B164" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7745,7 +7801,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B165" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7763,7 +7819,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B166" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7781,7 +7837,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B167" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7799,7 +7855,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B168" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7817,7 +7873,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B169" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7835,7 +7891,7 @@
         <v/>
       </c>
     </row>
-    <row r="170" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B170" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7853,7 +7909,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B171" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7871,7 +7927,7 @@
         <v/>
       </c>
     </row>
-    <row r="172" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B172" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7889,7 +7945,7 @@
         <v/>
       </c>
     </row>
-    <row r="173" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B173" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7907,7 +7963,7 @@
         <v/>
       </c>
     </row>
-    <row r="174" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B174" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7925,7 +7981,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B175" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7943,7 +7999,7 @@
         <v/>
       </c>
     </row>
-    <row r="176" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B176" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7961,7 +8017,7 @@
         <v/>
       </c>
     </row>
-    <row r="177" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B177" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7979,7 +8035,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B178" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7997,7 +8053,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B179" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8015,7 +8071,7 @@
         <v/>
       </c>
     </row>
-    <row r="180" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B180" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8033,7 +8089,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B181" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8051,7 +8107,7 @@
         <v/>
       </c>
     </row>
-    <row r="182" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B182" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8069,7 +8125,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B183" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8087,7 +8143,7 @@
         <v/>
       </c>
     </row>
-    <row r="184" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B184" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8105,7 +8161,7 @@
         <v/>
       </c>
     </row>
-    <row r="185" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B185" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8123,7 +8179,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B186" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8141,7 +8197,7 @@
         <v/>
       </c>
     </row>
-    <row r="187" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B187" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8159,7 +8215,7 @@
         <v/>
       </c>
     </row>
-    <row r="188" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B188" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8177,7 +8233,7 @@
         <v/>
       </c>
     </row>
-    <row r="189" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B189" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8195,7 +8251,7 @@
         <v/>
       </c>
     </row>
-    <row r="190" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B190" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8213,7 +8269,7 @@
         <v/>
       </c>
     </row>
-    <row r="191" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B191" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8231,7 +8287,7 @@
         <v/>
       </c>
     </row>
-    <row r="192" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B192" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8249,7 +8305,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B193" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8267,7 +8323,7 @@
         <v/>
       </c>
     </row>
-    <row r="194" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B194" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8285,7 +8341,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B195" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8303,7 +8359,7 @@
         <v/>
       </c>
     </row>
-    <row r="196" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B196" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8321,7 +8377,7 @@
         <v/>
       </c>
     </row>
-    <row r="197" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B197" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8339,7 +8395,7 @@
         <v/>
       </c>
     </row>
-    <row r="198" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B198" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8357,7 +8413,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B199" t="str">
         <f t="shared" ref="B199" si="15">IF(J199=0,"",J199)</f>
         <v/>
@@ -8382,112 +8438,84 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CF077CF-BCE9-46D4-AD95-5EB6BFB2C2E4}">
-  <dimension ref="B3:G13"/>
-  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:G17"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" s="68" t="s">
-        <v>134</v>
-      </c>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-    </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" s="69" t="s">
+    <row r="2" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B2" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="69" t="s">
+      <c r="C3" s="77" t="s">
+        <v>141</v>
+      </c>
+      <c r="D3" s="77" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B4" s="76" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="75" t="s">
+        <v>143</v>
+      </c>
+      <c r="D4" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="B5" s="76" t="s">
+        <v>142</v>
+      </c>
+      <c r="C5" s="75" t="s">
+        <v>144</v>
+      </c>
+      <c r="D5" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="68" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="68"/>
+      <c r="D7" s="68"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="69" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="69" t="s">
+      <c r="D8" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="69" t="s">
+      <c r="F8" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="G4" s="69" t="s">
+      <c r="G8" s="69" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" s="68" t="str">
-        <f t="shared" ref="B5:B11" si="0">IF(F5="Yes","RPT_OPT","*")</f>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="68" t="str">
+        <f t="shared" ref="B9:B15" si="0">IF(F9="Yes","RPT_OPT","*")</f>
         <v>*</v>
       </c>
-      <c r="C5" s="68" t="s">
+      <c r="C9" s="68" t="s">
         <v>103</v>
-      </c>
-      <c r="D5" s="68">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" s="68" t="str">
-        <f t="shared" si="0"/>
-        <v>RPT_OPT</v>
-      </c>
-      <c r="C6" s="68" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" s="68">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>107</v>
-      </c>
-      <c r="G6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="68" t="str">
-        <f t="shared" si="0"/>
-        <v>*</v>
-      </c>
-      <c r="C7" s="68" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" s="68">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
-        <v>104</v>
-      </c>
-      <c r="G7" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="68" t="str">
-        <f t="shared" si="0"/>
-        <v>*</v>
-      </c>
-      <c r="C8" s="68" t="s">
-        <v>111</v>
-      </c>
-      <c r="D8" s="68">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>104</v>
-      </c>
-      <c r="G8" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="68" t="str">
-        <f t="shared" si="0"/>
-        <v>*</v>
-      </c>
-      <c r="C9" s="68" t="s">
-        <v>113</v>
       </c>
       <c r="D9" s="68">
         <v>1</v>
@@ -8496,16 +8524,16 @@
         <v>104</v>
       </c>
       <c r="G9" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="68" t="str">
         <f t="shared" si="0"/>
         <v>RPT_OPT</v>
       </c>
       <c r="C10" s="68" t="s">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="D10" s="68">
         <v>1</v>
@@ -8514,31 +8542,103 @@
         <v>107</v>
       </c>
       <c r="G10" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="68" t="str">
         <f t="shared" si="0"/>
-        <v>RPT_OPT</v>
+        <v>*</v>
       </c>
       <c r="C11" s="68" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="D11" s="68">
         <v>1</v>
       </c>
       <c r="F11" t="s">
+        <v>104</v>
+      </c>
+      <c r="G11" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="68" t="str">
+        <f t="shared" si="0"/>
+        <v>*</v>
+      </c>
+      <c r="C12" s="68" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="68">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>104</v>
+      </c>
+      <c r="G12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="68" t="str">
+        <f t="shared" si="0"/>
+        <v>*</v>
+      </c>
+      <c r="C13" s="68" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" s="68">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>104</v>
+      </c>
+      <c r="G13" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="68" t="str">
+        <f t="shared" si="0"/>
+        <v>RPT_OPT</v>
+      </c>
+      <c r="C14" s="68" t="s">
+        <v>115</v>
+      </c>
+      <c r="D14" s="68">
+        <v>1</v>
+      </c>
+      <c r="F14" t="s">
         <v>107</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G14" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="68" t="str">
+        <f t="shared" si="0"/>
+        <v>RPT_OPT</v>
+      </c>
+      <c r="C15" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" s="68">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="68"/>
-      <c r="C13" s="68"/>
-      <c r="D13" s="68"/>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B17" s="68"/>
+      <c r="C17" s="68"/>
+      <c r="D17" s="68"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
README.md - Updated markdown documentation
Sets-DemoModels.xlsx -> Sets-DemoModels.xlsm: Change to makro-enabled workbook to automate the copying of proces and commodity sets to Scen_Z_TIMESReport.xlsx and SysSettings.xlsx.

Scen_Z_TIMESReport.xlsx -> Change how proces and commodity are written read by veda from a TFM_INS to TFM_DINS-AT (gives creater flexibility in terms of adding commas to the description of proces and commodity sets.

create_scen_desc_gms.bat -> improve the robustnes of reading and writing scenario description from the VTRUN.CMD file by moving this operation to "\GAMS_WrkTIMES\scenarioname\"-library.
</commit_message>
<xml_diff>
--- a/SysSettings.xlsx
+++ b/SysSettings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kristoffer\DemoS_012_timesreport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94DEBF54-460E-4CC8-BBA5-1028F83563E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C201E59-56E5-40B4-9506-9DA3F90491E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34670" yWindow="-110" windowWidth="34780" windowHeight="21100" tabRatio="853" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="57840" windowHeight="31920" tabRatio="853" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Region-Time Slices" sheetId="16" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Interpol_Extrapol_Defaults" sheetId="14" r:id="rId4"/>
     <sheet name="Constants" sheetId="20" r:id="rId5"/>
     <sheet name="Defaults" sheetId="21" r:id="rId6"/>
-    <sheet name="Commodity Group_TIMESreport" sheetId="15" r:id="rId7"/>
+    <sheet name="Commodity Group" sheetId="15" r:id="rId7"/>
     <sheet name="Runfile Switches" sheetId="23" r:id="rId8"/>
   </sheets>
   <externalReferences>
@@ -137,72 +137,11 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">The information in the table below is copied manually from the workbook Sets-DemoModels.xlsx, specifically from 'TIMESreport_Sets-Comm'!A2:C11.
+          <t xml:space="preserve">The information in the table below is copied using VBA-script in the the workbook Sets-DemoModels.xlsm, specifically from the range "TIMESreport_RangeCommoditySets"
 This is done because currently syssetting.xlsx and subres are the only files in VEDA that allow you to add information to the ~TFM_COMGRP.
 The role of ~TFM_COMGRP is that it adds the commodity sets so that they are available in the TIMES solution output file generated when solving the model in GAMS.
 By having information on commodity groups in the TIMES solution output file, we can access the information in the timesreport.gms script.
 </t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Note</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>: if you create additional commodity groups in Sets-DemoModels.xlsx, then you need to manually copy the new sets to syssetting.xlsx.</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <u/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Future improvement</t>
-        </r>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Perhaps a future version of VEDA could allow for the definition of TFM_COMGRP directly inside the Sets-DemoModels.xlsx. If this happens, then this step of timesreport could be skipped. </t>
         </r>
       </text>
     </comment>
@@ -576,6 +515,24 @@
     <t>TIMESReport</t>
   </si>
   <si>
+    <t>~TFM_COMGRP</t>
+  </si>
+  <si>
+    <t>GHG-emission</t>
+  </si>
+  <si>
+    <t>Other_indexes</t>
+  </si>
+  <si>
+    <t>RFCmd_FLAGS</t>
+  </si>
+  <si>
+    <t>$SET MEMCLEAN NO</t>
+  </si>
+  <si>
+    <t>$SET ANNCOST LEV</t>
+  </si>
+  <si>
     <t>NRG_ELC</t>
   </si>
   <si>
@@ -621,9 +578,6 @@
     <t>Biomass</t>
   </si>
   <si>
-    <t>~TFM_COMGRP</t>
-  </si>
-  <si>
     <t>ENV_CO2</t>
   </si>
   <si>
@@ -631,34 +585,18 @@
   </si>
   <si>
     <t>Demand commodity</t>
-  </si>
-  <si>
-    <t>GHG-emission</t>
-  </si>
-  <si>
-    <t>Other_indexes</t>
-  </si>
-  <si>
-    <t>RFCmd_FLAGS</t>
-  </si>
-  <si>
-    <t>$SET MEMCLEAN NO</t>
-  </si>
-  <si>
-    <t>$SET ANNCOST LEV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="165" formatCode="_([$€]* #,##0.00_);_([$€]* \(#,##0.00\);_([$€]* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="169" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="_([$€]* #,##0.00_);_([$€]* \(#,##0.00\);_([$€]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="31" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -770,6 +708,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -797,6 +736,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
@@ -816,28 +756,6 @@
       <family val="1"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
@@ -1132,7 +1050,7 @@
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
@@ -1151,7 +1069,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="17">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="4" fontId="24" fillId="0" borderId="0" applyBorder="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -1240,16 +1158,16 @@
     <xf numFmtId="0" fontId="16" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="4" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="4" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="4" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="4" borderId="9" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="4" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1346,7 +1264,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="30" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="30" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="30" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
@@ -3843,16 +3761,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:J6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.140625" customWidth="1"/>
-    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="3.42578125" customWidth="1"/>
-    <col min="8" max="8" width="29.42578125" customWidth="1"/>
+    <col min="1" max="1" width="2.15234375" customWidth="1"/>
+    <col min="2" max="2" width="19.15234375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.53515625" customWidth="1"/>
+    <col min="7" max="7" width="3.3828125" customWidth="1"/>
+    <col min="8" max="8" width="29.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3862,7 +3780,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
@@ -3879,7 +3797,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B5" s="15" t="s">
         <v>54</v>
       </c>
@@ -3893,7 +3811,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="15" t="s">
         <v>83</v>
       </c>
@@ -3920,42 +3838,42 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B3:D23"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.85546875" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.69140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.69140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.69140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.84375" customWidth="1"/>
+    <col min="6" max="6" width="8.69140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4">
         <v>2005</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B12" s="65" t="s">
         <v>40</v>
       </c>
@@ -3966,7 +3884,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B13" s="14">
         <v>1</v>
       </c>
@@ -3977,7 +3895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B14" s="14">
         <v>2</v>
       </c>
@@ -3988,7 +3906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B15" s="14"/>
       <c r="C15" s="14">
         <v>5</v>
@@ -3997,7 +3915,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B16" s="14"/>
       <c r="C16" s="14">
         <v>5</v>
@@ -4006,7 +3924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B17" s="14"/>
       <c r="C17" s="14">
         <v>5</v>
@@ -4015,42 +3933,42 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
       <c r="D22" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
       <c r="D23" s="14">
@@ -4069,18 +3987,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B3:C11"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.42578125" customWidth="1"/>
-    <col min="2" max="2" width="52.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.3828125" customWidth="1"/>
+    <col min="2" max="2" width="52.69140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="13" t="s">
         <v>32</v>
       </c>
@@ -4088,7 +4006,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="63" t="s">
         <v>34</v>
       </c>
@@ -4096,7 +4014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="14" t="s">
         <v>35</v>
       </c>
@@ -4104,7 +4022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" s="14" t="s">
         <v>36</v>
       </c>
@@ -4112,7 +4030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="14" t="s">
         <v>37</v>
       </c>
@@ -4120,7 +4038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="14" t="s">
         <v>98</v>
       </c>
@@ -4128,7 +4046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" s="14" t="s">
         <v>99</v>
       </c>
@@ -4136,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" s="14" t="s">
         <v>85</v>
       </c>
@@ -4156,23 +4074,23 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B3:Q36"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="2.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.7109375" customWidth="1"/>
-    <col min="13" max="13" width="9.28515625" customWidth="1"/>
+    <col min="1" max="1" width="2.84375" customWidth="1"/>
+    <col min="4" max="4" width="9.69140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.69140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.53515625" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.69140625" customWidth="1"/>
+    <col min="13" max="13" width="9.3046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>19</v>
       </c>
@@ -4192,7 +4110,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="C5" t="s">
         <v>86</v>
       </c>
@@ -4206,7 +4124,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
       <c r="C6" t="s">
         <v>86</v>
       </c>
@@ -4220,7 +4138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
       <c r="C7" t="s">
         <v>86</v>
       </c>
@@ -4234,26 +4152,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="2:4" ht="15" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="2:4" ht="15" x14ac:dyDescent="0.35">
       <c r="B30" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="2:4" ht="18" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:4" ht="17.600000000000001" x14ac:dyDescent="0.4">
       <c r="B32" s="8" t="s">
         <v>44</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:17" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="5" t="s">
         <v>19</v>
       </c>
@@ -4303,7 +4221,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:17" x14ac:dyDescent="0.3">
       <c r="D35" t="s">
         <v>4</v>
       </c>
@@ -4317,7 +4235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:17" x14ac:dyDescent="0.3">
       <c r="D36" t="s">
         <v>4</v>
       </c>
@@ -4343,28 +4261,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B3:H33"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="10"/>
-    <col min="2" max="2" width="12.140625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" style="10" customWidth="1"/>
+    <col min="1" max="1" width="9.15234375" style="10"/>
+    <col min="2" max="2" width="12.15234375" style="10" customWidth="1"/>
+    <col min="3" max="3" width="10.84375" style="10" customWidth="1"/>
     <col min="4" max="4" width="14" style="10" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" style="10" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="10"/>
+    <col min="5" max="5" width="10.3828125" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.3828125" style="10" customWidth="1"/>
+    <col min="7" max="16384" width="9.15234375" style="10"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:8" ht="15" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B5" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="5" t="s">
         <v>19</v>
       </c>
@@ -4387,7 +4305,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D7" s="10" t="s">
         <v>56</v>
       </c>
@@ -4395,7 +4313,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
       <c r="D8" s="10" t="s">
         <v>46</v>
       </c>
@@ -4403,7 +4321,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="10" t="s">
         <v>63</v>
       </c>
@@ -4415,7 +4333,7 @@
         <v>0.24971461187214614</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="10" t="s">
         <v>64</v>
       </c>
@@ -4427,7 +4345,7 @@
         <v>0.22973744292237441</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="10" t="s">
         <v>65</v>
       </c>
@@ -4439,7 +4357,7 @@
         <v>0.24942922374429224</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="10" t="s">
         <v>66</v>
       </c>
@@ -4451,7 +4369,7 @@
         <v>0.27111872146118721</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" s="10" t="s">
@@ -4467,34 +4385,34 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14"/>
       <c r="C14"/>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B15"/>
       <c r="C15"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B17"/>
       <c r="C17"/>
       <c r="D17"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18"/>
     </row>
-    <row r="19" spans="2:7" ht="18" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" ht="17.600000000000001" x14ac:dyDescent="0.4">
       <c r="B19" s="18" t="s">
         <v>62</v>
       </c>
@@ -4504,11 +4422,11 @@
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
       <c r="C20" s="21"/>
       <c r="D20" s="21"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B21" s="22" t="s">
         <v>21</v>
       </c>
@@ -4525,7 +4443,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="24" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B22" s="26"/>
       <c r="C22" s="27" t="s">
         <v>67</v>
@@ -4540,7 +4458,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B23" s="22" t="s">
         <v>55</v>
       </c>
@@ -4565,14 +4483,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" s="34"/>
       <c r="C24" s="34"/>
       <c r="D24" s="34"/>
       <c r="E24" s="34"/>
       <c r="F24" s="34"/>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B25" s="34"/>
       <c r="C25" s="35"/>
       <c r="D25" s="35"/>
@@ -4580,7 +4498,7 @@
       <c r="F25" s="34"/>
       <c r="G25" s="34"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B26" s="34"/>
       <c r="C26" s="36" t="s">
         <v>71</v>
@@ -4594,7 +4512,7 @@
       <c r="F26" s="39"/>
       <c r="G26" s="34"/>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B27" s="40" t="s">
         <v>74</v>
       </c>
@@ -4611,7 +4529,7 @@
       <c r="F27" s="44"/>
       <c r="G27" s="34"/>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B28" s="45" t="s">
         <v>76</v>
       </c>
@@ -4629,7 +4547,7 @@
       <c r="F28" s="44"/>
       <c r="G28" s="34"/>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B29" s="34"/>
       <c r="C29" s="34"/>
       <c r="D29" s="49">
@@ -4643,7 +4561,7 @@
       <c r="F29" s="51"/>
       <c r="G29" s="34"/>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B30" s="34"/>
       <c r="C30" s="34"/>
       <c r="D30" s="52"/>
@@ -4651,7 +4569,7 @@
       <c r="F30" s="34"/>
       <c r="G30" s="34"/>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B31" s="53"/>
       <c r="C31" s="54" t="s">
         <v>78</v>
@@ -4663,7 +4581,7 @@
       <c r="F31" s="34"/>
       <c r="G31" s="34"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B32" s="56" t="s">
         <v>75</v>
       </c>
@@ -4680,7 +4598,7 @@
       </c>
       <c r="G32" s="34"/>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B33" s="59" t="s">
         <v>80</v>
       </c>
@@ -4709,17 +4627,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:I6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.69140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.53515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.53515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.3046875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>48</v>
       </c>
@@ -4727,7 +4645,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:9" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="11" t="s">
         <v>49</v>
       </c>
@@ -4750,7 +4668,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B4" s="15" t="s">
         <v>97</v>
       </c>
@@ -4773,7 +4691,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D5" t="s">
         <v>52</v>
       </c>
@@ -4793,7 +4711,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
         <v>53</v>
       </c>
@@ -4823,18 +4741,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B2:L199"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.140625" customWidth="1"/>
-    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="3.15234375" customWidth="1"/>
+    <col min="2" max="2" width="15.69140625" customWidth="1"/>
     <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="11.28515625" customWidth="1"/>
-    <col min="9" max="11" width="11.85546875" customWidth="1"/>
+    <col min="4" max="4" width="8.69140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.3828125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.3046875" customWidth="1"/>
+    <col min="9" max="11" width="11.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:12" ht="15" x14ac:dyDescent="0.35">
       <c r="B2" s="6" t="s">
         <v>41</v>
       </c>
@@ -4845,7 +4763,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B4" s="8" t="s">
         <v>6</v>
       </c>
@@ -4854,12 +4772,12 @@
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
@@ -4879,7 +4797,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" ht="26.15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B7" s="70" t="s">
         <v>42</v>
       </c>
@@ -4900,7 +4818,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B8" t="str">
         <f t="shared" ref="B8:B13" si="0">IF(J8=0,"",J8)</f>
         <v>NRG_ELC</v>
@@ -4918,16 +4836,16 @@
         <v>y</v>
       </c>
       <c r="J8" s="71" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="K8" s="71" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="L8" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>NRG_GAS</v>
@@ -4944,16 +4862,16 @@
         <v>119</v>
       </c>
       <c r="J9" s="71" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="K9" s="71" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="L9" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>NRG_NUK</v>
@@ -4970,16 +4888,16 @@
         <v>119</v>
       </c>
       <c r="J10" s="71" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="K10" s="71" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="L10" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>NRG_OIL</v>
@@ -4996,16 +4914,16 @@
         <v>119</v>
       </c>
       <c r="J11" s="71" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="K11" s="71" t="s">
+        <v>135</v>
+      </c>
+      <c r="L11" s="71" t="s">
         <v>129</v>
       </c>
-      <c r="L11" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="12" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>NRG_RNW</v>
@@ -5022,16 +4940,16 @@
         <v>119</v>
       </c>
       <c r="J12" s="71" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="K12" s="71" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="L12" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="13" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>NRG_COA</v>
@@ -5048,16 +4966,16 @@
         <v>119</v>
       </c>
       <c r="J13" s="71" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="K13" s="71" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="L13" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="14" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B14" t="str">
         <f t="shared" ref="B14:B72" si="3">IF(J14=0,"",J14)</f>
         <v>NRG_BIO</v>
@@ -5075,22 +4993,22 @@
         <v>y</v>
       </c>
       <c r="J14" s="71" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="K14" s="71" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="L14" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="15" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B15" t="str">
         <f t="shared" si="3"/>
         <v>ENV_CO2</v>
       </c>
       <c r="C15" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="D15" t="str">
         <f t="shared" si="5"/>
@@ -5101,16 +5019,16 @@
         <v>y</v>
       </c>
       <c r="J15" s="71" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="K15" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="L15" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" ht="15" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B16" t="str">
         <f t="shared" si="3"/>
         <v>DEM_COM</v>
@@ -5128,16 +5046,16 @@
         <v>y</v>
       </c>
       <c r="J16" s="71" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="K16" s="71" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="L16" s="71" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B17" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5155,7 +5073,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B18" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5173,7 +5091,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B19" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5191,7 +5109,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B20" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5209,7 +5127,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B21" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5227,7 +5145,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B22" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5245,7 +5163,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5263,7 +5181,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5281,7 +5199,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B25" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5299,7 +5217,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B26" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5317,7 +5235,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B27" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5335,7 +5253,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B28" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5353,7 +5271,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B29" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5371,7 +5289,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B30" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5389,7 +5307,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B31" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5407,7 +5325,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B32" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5425,7 +5343,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B33" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5443,7 +5361,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B34" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5461,7 +5379,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B35" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5479,7 +5397,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B36" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5497,7 +5415,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B37" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5515,7 +5433,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B38" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5533,7 +5451,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B39" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5551,7 +5469,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5569,7 +5487,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B41" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5587,7 +5505,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B42" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5605,7 +5523,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B43" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5623,7 +5541,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B44" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5641,7 +5559,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B45" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5659,7 +5577,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B46" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5677,7 +5595,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B47" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5695,7 +5613,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B48" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5713,7 +5631,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B49" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5731,7 +5649,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B50" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5749,7 +5667,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B51" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5767,7 +5685,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B52" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5785,7 +5703,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B53" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5803,7 +5721,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B54" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5821,7 +5739,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B55" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5839,7 +5757,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B56" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5857,7 +5775,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B57" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5875,7 +5793,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B58" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5893,7 +5811,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B59" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5911,7 +5829,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B60" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5929,7 +5847,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B61" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5947,7 +5865,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B62" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5965,7 +5883,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B63" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5983,7 +5901,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B64" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6001,7 +5919,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B65" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6019,7 +5937,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B66" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6037,7 +5955,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B67" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6055,7 +5973,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B68" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6073,7 +5991,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B69" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6091,7 +6009,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B70" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6109,7 +6027,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B71" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6127,7 +6045,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B72" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6145,7 +6063,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B73" t="str">
         <f t="shared" ref="B73:B136" si="7">IF(J73=0,"",J73)</f>
         <v/>
@@ -6163,7 +6081,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B74" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6181,7 +6099,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B75" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6199,7 +6117,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B76" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6217,7 +6135,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B77" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6235,7 +6153,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B78" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6253,7 +6171,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B79" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6271,7 +6189,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B80" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6289,7 +6207,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B81" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6307,7 +6225,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B82" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6325,7 +6243,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B83" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6343,7 +6261,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B84" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6361,7 +6279,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B85" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6379,7 +6297,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B86" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6397,7 +6315,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B87" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6415,7 +6333,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B88" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6433,7 +6351,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B89" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6451,7 +6369,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B90" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6469,7 +6387,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B91" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6487,7 +6405,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B92" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6505,7 +6423,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B93" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6523,7 +6441,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B94" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6541,7 +6459,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B95" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6559,7 +6477,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B96" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6577,7 +6495,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B97" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6595,7 +6513,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B98" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6613,7 +6531,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B99" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6631,7 +6549,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B100" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6649,7 +6567,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B101" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6667,7 +6585,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B102" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6685,7 +6603,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B103" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6703,7 +6621,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B104" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6721,7 +6639,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B105" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6739,7 +6657,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B106" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6757,7 +6675,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B107" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6775,7 +6693,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B108" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6793,7 +6711,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B109" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6811,7 +6729,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B110" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6829,7 +6747,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B111" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6847,7 +6765,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B112" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6865,7 +6783,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B113" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6883,7 +6801,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B114" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6901,7 +6819,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B115" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6919,7 +6837,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B116" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6937,7 +6855,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B117" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6955,7 +6873,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B118" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6973,7 +6891,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B119" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6991,7 +6909,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B120" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7009,7 +6927,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B121" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7027,7 +6945,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B122" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7045,7 +6963,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B123" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7063,7 +6981,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B124" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7081,7 +6999,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B125" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7099,7 +7017,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B126" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7117,7 +7035,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B127" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7135,7 +7053,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B128" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7153,7 +7071,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B129" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7171,7 +7089,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B130" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7189,7 +7107,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B131" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7207,7 +7125,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B132" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7225,7 +7143,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B133" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7243,7 +7161,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B134" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7261,7 +7179,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B135" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7279,7 +7197,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B136" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7297,7 +7215,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B137" t="str">
         <f t="shared" ref="B137:B198" si="11">IF(J137=0,"",J137)</f>
         <v/>
@@ -7315,7 +7233,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B138" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7333,7 +7251,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B139" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7351,7 +7269,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B140" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7369,7 +7287,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B141" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7387,7 +7305,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B142" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7405,7 +7323,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B143" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7423,7 +7341,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B144" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7441,7 +7359,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B145" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7459,7 +7377,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B146" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7477,7 +7395,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B147" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7495,7 +7413,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B148" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7513,7 +7431,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B149" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7531,7 +7449,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B150" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7549,7 +7467,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B151" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7567,7 +7485,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B152" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7585,7 +7503,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B153" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7603,7 +7521,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B154" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7621,7 +7539,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B155" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7639,7 +7557,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B156" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7657,7 +7575,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B157" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7675,7 +7593,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B158" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7693,7 +7611,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B159" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7711,7 +7629,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="160" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B160" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7729,7 +7647,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B161" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7747,7 +7665,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B162" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7765,7 +7683,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B163" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7783,7 +7701,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B164" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7801,7 +7719,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B165" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7819,7 +7737,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B166" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7837,7 +7755,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B167" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7855,7 +7773,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="168" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B168" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7873,7 +7791,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B169" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7891,7 +7809,7 @@
         <v/>
       </c>
     </row>
-    <row r="170" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B170" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7909,7 +7827,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B171" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7927,7 +7845,7 @@
         <v/>
       </c>
     </row>
-    <row r="172" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B172" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7945,7 +7863,7 @@
         <v/>
       </c>
     </row>
-    <row r="173" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B173" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7963,7 +7881,7 @@
         <v/>
       </c>
     </row>
-    <row r="174" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="174" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B174" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7981,7 +7899,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B175" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7999,7 +7917,7 @@
         <v/>
       </c>
     </row>
-    <row r="176" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B176" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8017,7 +7935,7 @@
         <v/>
       </c>
     </row>
-    <row r="177" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B177" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8035,7 +7953,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B178" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8053,7 +7971,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="179" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B179" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8071,7 +7989,7 @@
         <v/>
       </c>
     </row>
-    <row r="180" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="180" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B180" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8089,7 +8007,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B181" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8107,7 +8025,7 @@
         <v/>
       </c>
     </row>
-    <row r="182" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B182" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8125,7 +8043,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="183" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B183" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8143,7 +8061,7 @@
         <v/>
       </c>
     </row>
-    <row r="184" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B184" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8161,7 +8079,7 @@
         <v/>
       </c>
     </row>
-    <row r="185" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B185" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8179,7 +8097,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B186" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8197,7 +8115,7 @@
         <v/>
       </c>
     </row>
-    <row r="187" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B187" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8215,7 +8133,7 @@
         <v/>
       </c>
     </row>
-    <row r="188" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="188" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B188" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8233,7 +8151,7 @@
         <v/>
       </c>
     </row>
-    <row r="189" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B189" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8251,7 +8169,7 @@
         <v/>
       </c>
     </row>
-    <row r="190" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B190" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8269,7 +8187,7 @@
         <v/>
       </c>
     </row>
-    <row r="191" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B191" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8287,7 +8205,7 @@
         <v/>
       </c>
     </row>
-    <row r="192" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="192" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B192" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8305,7 +8223,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="193" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B193" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8323,7 +8241,7 @@
         <v/>
       </c>
     </row>
-    <row r="194" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="194" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B194" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8341,7 +8259,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="195" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B195" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8359,7 +8277,7 @@
         <v/>
       </c>
     </row>
-    <row r="196" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="196" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B196" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8377,7 +8295,7 @@
         <v/>
       </c>
     </row>
-    <row r="197" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="197" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B197" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8395,7 +8313,7 @@
         <v/>
       </c>
     </row>
-    <row r="198" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="198" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B198" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8413,7 +8331,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="199" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B199" t="str">
         <f t="shared" ref="B199" si="15">IF(J199=0,"",J199)</f>
         <v/>
@@ -8439,60 +8357,60 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CF077CF-BCE9-46D4-AD95-5EB6BFB2C2E4}">
   <dimension ref="B2:G17"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
-    <col min="3" max="3" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.15234375" customWidth="1"/>
+    <col min="3" max="3" width="22.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B2" s="74" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="73"/>
       <c r="D2" s="73"/>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B3" s="77" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="D3" s="77" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B4" s="76" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="C4" s="75" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
       <c r="D4" s="73">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="15" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:7" ht="14.6" x14ac:dyDescent="0.4">
       <c r="B5" s="76" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="C5" s="75" t="s">
-        <v>144</v>
+        <v>126</v>
       </c>
       <c r="D5" s="73">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B7" s="68" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="68"/>
       <c r="D7" s="68"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B8" s="69" t="s">
         <v>21</v>
       </c>
@@ -8509,7 +8427,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B9" s="68" t="str">
         <f t="shared" ref="B9:B15" si="0">IF(F9="Yes","RPT_OPT","*")</f>
         <v>*</v>
@@ -8527,7 +8445,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B10" s="68" t="str">
         <f t="shared" si="0"/>
         <v>RPT_OPT</v>
@@ -8545,7 +8463,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B11" s="68" t="str">
         <f t="shared" si="0"/>
         <v>*</v>
@@ -8563,7 +8481,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B12" s="68" t="str">
         <f t="shared" si="0"/>
         <v>*</v>
@@ -8581,7 +8499,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B13" s="68" t="str">
         <f t="shared" si="0"/>
         <v>*</v>
@@ -8599,7 +8517,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B14" s="68" t="str">
         <f t="shared" si="0"/>
         <v>RPT_OPT</v>
@@ -8617,7 +8535,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B15" s="68" t="str">
         <f t="shared" si="0"/>
         <v>RPT_OPT</v>
@@ -8635,7 +8553,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B17" s="68"/>
       <c r="C17" s="68"/>
       <c r="D17" s="68"/>

</xml_diff>

<commit_message>
Corrected error in create_times_db_multiple_scenarios.R related to install.packages and related to library issues.
</commit_message>
<xml_diff>
--- a/SysSettings.xlsx
+++ b/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kristoffer\DemoS_012_timesreport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C201E59-56E5-40B4-9506-9DA3F90491E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A986E05F-4C5E-4559-AB3F-0C672C18DB95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="57840" windowHeight="31920" tabRatio="853" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="853" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Region-Time Slices" sheetId="16" r:id="rId1"/>
@@ -3761,16 +3761,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:J6"/>
-  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.15234375" customWidth="1"/>
-    <col min="2" max="2" width="19.15234375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.53515625" customWidth="1"/>
-    <col min="7" max="7" width="3.3828125" customWidth="1"/>
-    <col min="8" max="8" width="29.3828125" customWidth="1"/>
+    <col min="1" max="1" width="2.140625" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="3.42578125" customWidth="1"/>
+    <col min="8" max="8" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3780,7 +3780,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
@@ -3797,7 +3797,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B5" s="15" t="s">
         <v>54</v>
       </c>
@@ -3811,7 +3811,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B6" s="15" t="s">
         <v>83</v>
       </c>
@@ -3838,42 +3838,42 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B3:D23"/>
-  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="13.69140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.69140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.69140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.84375" customWidth="1"/>
-    <col min="6" max="6" width="8.69140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4">
         <v>2005</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B12" s="65" t="s">
         <v>40</v>
       </c>
@@ -3884,7 +3884,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B13" s="14">
         <v>1</v>
       </c>
@@ -3895,7 +3895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B14" s="14">
         <v>2</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B15" s="14"/>
       <c r="C15" s="14">
         <v>5</v>
@@ -3915,7 +3915,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B16" s="14"/>
       <c r="C16" s="14">
         <v>5</v>
@@ -3924,7 +3924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="14"/>
       <c r="C17" s="14">
         <v>5</v>
@@ -3933,42 +3933,42 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
       <c r="D20" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
       <c r="D22" s="14">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
       <c r="D23" s="14">
@@ -3987,18 +3987,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B3:C11"/>
-  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.3828125" customWidth="1"/>
-    <col min="2" max="2" width="52.69140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.42578125" customWidth="1"/>
+    <col min="2" max="2" width="52.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="13" t="s">
         <v>32</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="63" t="s">
         <v>34</v>
       </c>
@@ -4014,7 +4014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="14" t="s">
         <v>35</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="14" t="s">
         <v>36</v>
       </c>
@@ -4030,7 +4030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="14" t="s">
         <v>37</v>
       </c>
@@ -4038,7 +4038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="14" t="s">
         <v>98</v>
       </c>
@@ -4046,7 +4046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="14" t="s">
         <v>99</v>
       </c>
@@ -4054,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="14" t="s">
         <v>85</v>
       </c>
@@ -4074,23 +4074,23 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B3:Q36"/>
-  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="2.84375" customWidth="1"/>
-    <col min="4" max="4" width="9.69140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.69140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.53515625" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="10.69140625" customWidth="1"/>
-    <col min="13" max="13" width="9.3046875" customWidth="1"/>
+    <col min="1" max="1" width="2.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="10.7109375" customWidth="1"/>
+    <col min="13" max="13" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>19</v>
       </c>
@@ -4110,7 +4110,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
         <v>86</v>
       </c>
@@ -4124,7 +4124,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C6" t="s">
         <v>86</v>
       </c>
@@ -4138,7 +4138,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>86</v>
       </c>
@@ -4152,26 +4152,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="2:4" ht="15" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="2:4" ht="15" x14ac:dyDescent="0.2">
       <c r="B30" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="32" spans="2:4" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:4" ht="18" x14ac:dyDescent="0.25">
       <c r="B32" s="8" t="s">
         <v>44</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B33" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:17" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:17" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B34" s="5" t="s">
         <v>19</v>
       </c>
@@ -4221,7 +4221,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:17" x14ac:dyDescent="0.2">
       <c r="D35" t="s">
         <v>4</v>
       </c>
@@ -4235,7 +4235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:17" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
         <v>4</v>
       </c>
@@ -4261,28 +4261,28 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B3:H33"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.15234375" style="10"/>
-    <col min="2" max="2" width="12.15234375" style="10" customWidth="1"/>
-    <col min="3" max="3" width="10.84375" style="10" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="10"/>
+    <col min="2" max="2" width="12.140625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" style="10" customWidth="1"/>
     <col min="4" max="4" width="14" style="10" customWidth="1"/>
-    <col min="5" max="5" width="10.3828125" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.3828125" style="10" customWidth="1"/>
-    <col min="7" max="16384" width="9.15234375" style="10"/>
+    <col min="5" max="5" width="10.42578125" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="10" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="10"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" ht="15" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" ht="15" x14ac:dyDescent="0.2">
       <c r="B3" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B5" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>19</v>
       </c>
@@ -4305,7 +4305,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
       <c r="D7" s="10" t="s">
         <v>56</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>2005</v>
       </c>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
       <c r="D8" s="10" t="s">
         <v>46</v>
       </c>
@@ -4321,7 +4321,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>63</v>
       </c>
@@ -4333,7 +4333,7 @@
         <v>0.24971461187214614</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B10" s="10" t="s">
         <v>64</v>
       </c>
@@ -4345,7 +4345,7 @@
         <v>0.22973744292237441</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B11" s="10" t="s">
         <v>65</v>
       </c>
@@ -4357,7 +4357,7 @@
         <v>0.24942922374429224</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B12" s="10" t="s">
         <v>66</v>
       </c>
@@ -4369,7 +4369,7 @@
         <v>0.27111872146118721</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" s="10" t="s">
@@ -4385,34 +4385,34 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B14"/>
       <c r="C14"/>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B15"/>
       <c r="C15"/>
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17"/>
       <c r="C17"/>
       <c r="D17"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18"/>
     </row>
-    <row r="19" spans="2:7" ht="17.600000000000001" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:7" ht="18" x14ac:dyDescent="0.25">
       <c r="B19" s="18" t="s">
         <v>62</v>
       </c>
@@ -4422,11 +4422,11 @@
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C20" s="21"/>
       <c r="D20" s="21"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="22" t="s">
         <v>21</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:7" ht="24" x14ac:dyDescent="0.2">
       <c r="B22" s="26"/>
       <c r="C22" s="27" t="s">
         <v>67</v>
@@ -4458,7 +4458,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="22" t="s">
         <v>55</v>
       </c>
@@ -4483,14 +4483,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="34"/>
       <c r="C24" s="34"/>
       <c r="D24" s="34"/>
       <c r="E24" s="34"/>
       <c r="F24" s="34"/>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" s="34"/>
       <c r="C25" s="35"/>
       <c r="D25" s="35"/>
@@ -4498,7 +4498,7 @@
       <c r="F25" s="34"/>
       <c r="G25" s="34"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="34"/>
       <c r="C26" s="36" t="s">
         <v>71</v>
@@ -4512,7 +4512,7 @@
       <c r="F26" s="39"/>
       <c r="G26" s="34"/>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" s="40" t="s">
         <v>74</v>
       </c>
@@ -4529,7 +4529,7 @@
       <c r="F27" s="44"/>
       <c r="G27" s="34"/>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="45" t="s">
         <v>76</v>
       </c>
@@ -4547,7 +4547,7 @@
       <c r="F28" s="44"/>
       <c r="G28" s="34"/>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" s="34"/>
       <c r="C29" s="34"/>
       <c r="D29" s="49">
@@ -4561,7 +4561,7 @@
       <c r="F29" s="51"/>
       <c r="G29" s="34"/>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="34"/>
       <c r="C30" s="34"/>
       <c r="D30" s="52"/>
@@ -4569,7 +4569,7 @@
       <c r="F30" s="34"/>
       <c r="G30" s="34"/>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" s="53"/>
       <c r="C31" s="54" t="s">
         <v>78</v>
@@ -4581,7 +4581,7 @@
       <c r="F31" s="34"/>
       <c r="G31" s="34"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="56" t="s">
         <v>75</v>
       </c>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="G32" s="34"/>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" s="59" t="s">
         <v>80</v>
       </c>
@@ -4627,17 +4627,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B2:I6"/>
-  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="11.69140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.53515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.53515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.3046875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
         <v>48</v>
       </c>
@@ -4645,7 +4645,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="12.9" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B3" s="11" t="s">
         <v>49</v>
       </c>
@@ -4668,7 +4668,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B4" s="15" t="s">
         <v>97</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
       <c r="D5" t="s">
         <v>52</v>
       </c>
@@ -4711,7 +4711,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
       <c r="D6" t="s">
         <v>53</v>
       </c>
@@ -4741,18 +4741,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="B2:L199"/>
-  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.15234375" customWidth="1"/>
-    <col min="2" max="2" width="15.69140625" customWidth="1"/>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
     <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.69140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.3828125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="11.3046875" customWidth="1"/>
-    <col min="9" max="11" width="11.84375" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.28515625" customWidth="1"/>
+    <col min="9" max="11" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="15" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:12" ht="15" x14ac:dyDescent="0.2">
       <c r="B2" s="6" t="s">
         <v>41</v>
       </c>
@@ -4763,7 +4763,7 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
     </row>
-    <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="8" t="s">
         <v>6</v>
       </c>
@@ -4772,12 +4772,12 @@
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
     </row>
-    <row r="5" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:12" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
@@ -4797,7 +4797,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:12" ht="26.15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:12" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="70" t="s">
         <v>42</v>
       </c>
@@ -4818,7 +4818,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B8" t="str">
         <f t="shared" ref="B8:B13" si="0">IF(J8=0,"",J8)</f>
         <v>NRG_ELC</v>
@@ -4845,7 +4845,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>NRG_GAS</v>
@@ -4871,7 +4871,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>NRG_NUK</v>
@@ -4897,7 +4897,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>NRG_OIL</v>
@@ -4923,7 +4923,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="12" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>NRG_RNW</v>
@@ -4949,7 +4949,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>NRG_COA</v>
@@ -4975,7 +4975,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="14" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f t="shared" ref="B14:B72" si="3">IF(J14=0,"",J14)</f>
         <v>NRG_BIO</v>
@@ -5002,7 +5002,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="15" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f t="shared" si="3"/>
         <v>ENV_CO2</v>
@@ -5028,7 +5028,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="2:12" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:12" ht="15" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f t="shared" si="3"/>
         <v>DEM_COM</v>
@@ -5055,7 +5055,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5073,7 +5073,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5091,7 +5091,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5109,7 +5109,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5127,7 +5127,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5145,7 +5145,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5163,7 +5163,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5181,7 +5181,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5199,7 +5199,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B25" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5217,7 +5217,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5235,7 +5235,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B27" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5253,7 +5253,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5271,7 +5271,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B29" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5289,7 +5289,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5307,7 +5307,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B31" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5325,7 +5325,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5343,7 +5343,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B33" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B34" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5379,7 +5379,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5397,7 +5397,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B36" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5415,7 +5415,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5433,7 +5433,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B38" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5451,7 +5451,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5469,7 +5469,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B40" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5487,7 +5487,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5505,7 +5505,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B42" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5523,7 +5523,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5541,7 +5541,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B44" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5559,7 +5559,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B45" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5577,7 +5577,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B46" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5595,7 +5595,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B47" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5613,7 +5613,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B48" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5631,7 +5631,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B49" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5649,7 +5649,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B50" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5667,7 +5667,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B51" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5685,7 +5685,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B52" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5703,7 +5703,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B53" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5721,7 +5721,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B54" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5739,7 +5739,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B55" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5757,7 +5757,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B56" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5775,7 +5775,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B57" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5793,7 +5793,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B58" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5811,7 +5811,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B59" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5829,7 +5829,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B60" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5847,7 +5847,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B61" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5865,7 +5865,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B62" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5883,7 +5883,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B63" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5901,7 +5901,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B64" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5919,7 +5919,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B65" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5937,7 +5937,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B66" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5955,7 +5955,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B67" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5973,7 +5973,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B68" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5991,7 +5991,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B69" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6009,7 +6009,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B70" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6027,7 +6027,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B71" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6045,7 +6045,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B72" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6063,7 +6063,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B73" t="str">
         <f t="shared" ref="B73:B136" si="7">IF(J73=0,"",J73)</f>
         <v/>
@@ -6081,7 +6081,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B74" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6099,7 +6099,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B75" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6117,7 +6117,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B76" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6135,7 +6135,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B77" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6153,7 +6153,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B78" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6171,7 +6171,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B79" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6189,7 +6189,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B80" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6207,7 +6207,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B81" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6225,7 +6225,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B82" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6243,7 +6243,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B83" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6261,7 +6261,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B84" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6279,7 +6279,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B85" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6297,7 +6297,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B86" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B87" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6333,7 +6333,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B88" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6351,7 +6351,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B89" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6369,7 +6369,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B90" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6387,7 +6387,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B91" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6405,7 +6405,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B92" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6423,7 +6423,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B93" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6441,7 +6441,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B94" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6459,7 +6459,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B95" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6477,7 +6477,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B96" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6495,7 +6495,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B97" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6513,7 +6513,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B98" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6531,7 +6531,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B99" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6549,7 +6549,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B100" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6567,7 +6567,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B101" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6585,7 +6585,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B102" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6603,7 +6603,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B103" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6621,7 +6621,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B104" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6639,7 +6639,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B105" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6657,7 +6657,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B106" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6675,7 +6675,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B107" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6693,7 +6693,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B108" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6711,7 +6711,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B109" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6729,7 +6729,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B110" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6747,7 +6747,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B111" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6765,7 +6765,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B112" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6783,7 +6783,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B113" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6801,7 +6801,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B114" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6819,7 +6819,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B115" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6837,7 +6837,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B116" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6855,7 +6855,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B117" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6873,7 +6873,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B118" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6891,7 +6891,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B119" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6909,7 +6909,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B120" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6927,7 +6927,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B121" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6945,7 +6945,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B122" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6963,7 +6963,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B123" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6981,7 +6981,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B124" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -6999,7 +6999,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B125" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7017,7 +7017,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B126" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7035,7 +7035,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B127" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7053,7 +7053,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B128" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7071,7 +7071,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B129" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7089,7 +7089,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B130" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7107,7 +7107,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B131" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7125,7 +7125,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B132" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7143,7 +7143,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B133" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7161,7 +7161,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B134" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7179,7 +7179,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B135" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7197,7 +7197,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B136" t="str">
         <f t="shared" si="7"/>
         <v/>
@@ -7215,7 +7215,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B137" t="str">
         <f t="shared" ref="B137:B198" si="11">IF(J137=0,"",J137)</f>
         <v/>
@@ -7233,7 +7233,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B138" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7251,7 +7251,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B139" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7269,7 +7269,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B140" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7287,7 +7287,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B141" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7305,7 +7305,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B142" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7323,7 +7323,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B143" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7341,7 +7341,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B144" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7359,7 +7359,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B145" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7377,7 +7377,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B146" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7395,7 +7395,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B147" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7413,7 +7413,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B148" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7431,7 +7431,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B149" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7449,7 +7449,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B150" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7467,7 +7467,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B151" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7485,7 +7485,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B152" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7503,7 +7503,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B153" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7521,7 +7521,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B154" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7539,7 +7539,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B155" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7557,7 +7557,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="156" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B156" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7575,7 +7575,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="157" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B157" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7593,7 +7593,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="158" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B158" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7611,7 +7611,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="159" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B159" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7629,7 +7629,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="160" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B160" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7647,7 +7647,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="161" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B161" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7665,7 +7665,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="162" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B162" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7683,7 +7683,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="163" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B163" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7701,7 +7701,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="164" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B164" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7719,7 +7719,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="165" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B165" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7737,7 +7737,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="166" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B166" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7755,7 +7755,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="167" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B167" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7773,7 +7773,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="168" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B168" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7791,7 +7791,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="169" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B169" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7809,7 +7809,7 @@
         <v/>
       </c>
     </row>
-    <row r="170" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="170" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B170" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7827,7 +7827,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="171" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B171" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7845,7 +7845,7 @@
         <v/>
       </c>
     </row>
-    <row r="172" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="172" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B172" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7863,7 +7863,7 @@
         <v/>
       </c>
     </row>
-    <row r="173" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="173" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B173" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7881,7 +7881,7 @@
         <v/>
       </c>
     </row>
-    <row r="174" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="174" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B174" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7899,7 +7899,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="175" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B175" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7917,7 +7917,7 @@
         <v/>
       </c>
     </row>
-    <row r="176" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="176" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B176" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7935,7 +7935,7 @@
         <v/>
       </c>
     </row>
-    <row r="177" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="177" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B177" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7953,7 +7953,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="178" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B178" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7971,7 +7971,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="179" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B179" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -7989,7 +7989,7 @@
         <v/>
       </c>
     </row>
-    <row r="180" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="180" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B180" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8007,7 +8007,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="181" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B181" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8025,7 +8025,7 @@
         <v/>
       </c>
     </row>
-    <row r="182" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="182" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B182" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8043,7 +8043,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="183" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B183" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8061,7 +8061,7 @@
         <v/>
       </c>
     </row>
-    <row r="184" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="184" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B184" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8079,7 +8079,7 @@
         <v/>
       </c>
     </row>
-    <row r="185" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="185" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B185" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8097,7 +8097,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="186" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B186" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8115,7 +8115,7 @@
         <v/>
       </c>
     </row>
-    <row r="187" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="187" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B187" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8133,7 +8133,7 @@
         <v/>
       </c>
     </row>
-    <row r="188" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="188" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B188" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8151,7 +8151,7 @@
         <v/>
       </c>
     </row>
-    <row r="189" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="189" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B189" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8169,7 +8169,7 @@
         <v/>
       </c>
     </row>
-    <row r="190" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="190" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B190" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8187,7 +8187,7 @@
         <v/>
       </c>
     </row>
-    <row r="191" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="191" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B191" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8205,7 +8205,7 @@
         <v/>
       </c>
     </row>
-    <row r="192" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="192" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B192" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8223,7 +8223,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="193" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B193" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8241,7 +8241,7 @@
         <v/>
       </c>
     </row>
-    <row r="194" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="194" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B194" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8259,7 +8259,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="195" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B195" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8277,7 +8277,7 @@
         <v/>
       </c>
     </row>
-    <row r="196" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="196" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B196" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8295,7 +8295,7 @@
         <v/>
       </c>
     </row>
-    <row r="197" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="197" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B197" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8313,7 +8313,7 @@
         <v/>
       </c>
     </row>
-    <row r="198" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="198" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B198" t="str">
         <f t="shared" si="11"/>
         <v/>
@@ -8331,7 +8331,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="199" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B199" t="str">
         <f t="shared" ref="B199" si="15">IF(J199=0,"",J199)</f>
         <v/>
@@ -8357,20 +8357,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CF077CF-BCE9-46D4-AD95-5EB6BFB2C2E4}">
   <dimension ref="B2:G17"/>
-  <sheetFormatPr defaultRowHeight="12.45" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="18.15234375" customWidth="1"/>
-    <col min="3" max="3" width="22.69140625" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:7" ht="15" x14ac:dyDescent="0.25">
       <c r="B2" s="74" t="s">
         <v>18</v>
       </c>
       <c r="C2" s="73"/>
       <c r="D2" s="73"/>
     </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="77" t="s">
         <v>21</v>
       </c>
@@ -8381,7 +8381,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:7" ht="15" x14ac:dyDescent="0.25">
       <c r="B4" s="76" t="s">
         <v>124</v>
       </c>
@@ -8392,7 +8392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="14.6" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:7" ht="15" x14ac:dyDescent="0.25">
       <c r="B5" s="76" t="s">
         <v>124</v>
       </c>
@@ -8403,14 +8403,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B7" s="68" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="68"/>
       <c r="D7" s="68"/>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="69" t="s">
         <v>21</v>
       </c>
@@ -8427,7 +8427,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B9" s="68" t="str">
         <f t="shared" ref="B9:B15" si="0">IF(F9="Yes","RPT_OPT","*")</f>
         <v>*</v>
@@ -8445,7 +8445,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="68" t="str">
         <f t="shared" si="0"/>
         <v>RPT_OPT</v>
@@ -8463,7 +8463,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B11" s="68" t="str">
         <f t="shared" si="0"/>
         <v>*</v>
@@ -8481,7 +8481,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="68" t="str">
         <f t="shared" si="0"/>
         <v>*</v>
@@ -8499,7 +8499,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B13" s="68" t="str">
         <f t="shared" si="0"/>
         <v>*</v>
@@ -8517,7 +8517,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="68" t="str">
         <f t="shared" si="0"/>
         <v>RPT_OPT</v>
@@ -8535,7 +8535,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B15" s="68" t="str">
         <f t="shared" si="0"/>
         <v>RPT_OPT</v>
@@ -8553,7 +8553,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B17" s="68"/>
       <c r="C17" s="68"/>
       <c r="D17" s="68"/>

</xml_diff>